<commit_message>
Added notes on pipeline IO, questions about data.
</commit_message>
<xml_diff>
--- a/data_sync/gasdermin/2025-07-26_gasdermin_annotated.xlsx
+++ b/data_sync/gasdermin/2025-07-26_gasdermin_annotated.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29122"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="25" documentId="11_1151F84A935E320F62355476585DCE3A87421C02" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B46EDAF-D0E9-46C1-9B0C-FAC7C5B64AF5}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\juliandeanmoran\___git_repos\BISSH\data_sync\gasdermin\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2416AAA1-3031-42FE-8DB5-0B2B7AE1DE45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1585,7 +1590,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2016,20 +2021,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BR77"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="11.28515625" customWidth="1"/>
-    <col min="3" max="3" width="11.85546875" customWidth="1"/>
-    <col min="4" max="4" width="21.42578125" customWidth="1"/>
-    <col min="5" max="5" width="12.5703125" customWidth="1"/>
-    <col min="10" max="10" width="14.85546875" customWidth="1"/>
-    <col min="11" max="11" width="15.28515625" customWidth="1"/>
-    <col min="52" max="52" width="9.5703125" customWidth="1"/>
-    <col min="69" max="69" width="12.85546875" customWidth="1"/>
+    <col min="2" max="2" width="11.26953125" customWidth="1"/>
+    <col min="3" max="3" width="11.81640625" customWidth="1"/>
+    <col min="4" max="4" width="21.453125" customWidth="1"/>
+    <col min="5" max="5" width="12.54296875" customWidth="1"/>
+    <col min="10" max="10" width="14.81640625" customWidth="1"/>
+    <col min="11" max="11" width="15.26953125" customWidth="1"/>
+    <col min="52" max="52" width="9.54296875" customWidth="1"/>
+    <col min="69" max="69" width="12.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:70">
+    <row r="1" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -2115,7 +2120,7 @@
       <c r="BQ1" s="3"/>
       <c r="BR1" s="3"/>
     </row>
-    <row r="2" spans="1:70" s="2" customFormat="1" ht="76.5">
+    <row r="2" spans="1:70" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -2327,7 +2332,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="3" spans="1:70">
+    <row r="3" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>77</v>
       </c>
@@ -2425,7 +2430,7 @@
         <v>0.95104895104895104</v>
       </c>
     </row>
-    <row r="4" spans="1:70">
+    <row r="4" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>77</v>
       </c>
@@ -2571,7 +2576,7 @@
         <v>0.96153846153846156</v>
       </c>
     </row>
-    <row r="5" spans="1:70">
+    <row r="5" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>77</v>
       </c>
@@ -2732,7 +2737,7 @@
         <v>0.76573426573426573</v>
       </c>
     </row>
-    <row r="6" spans="1:70">
+    <row r="6" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>77</v>
       </c>
@@ -2887,7 +2892,7 @@
         <v>0.95804195804195802</v>
       </c>
     </row>
-    <row r="7" spans="1:70">
+    <row r="7" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>77</v>
       </c>
@@ -3057,7 +3062,7 @@
         <v>0.97202797202797198</v>
       </c>
     </row>
-    <row r="8" spans="1:70">
+    <row r="8" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>77</v>
       </c>
@@ -3212,7 +3217,7 @@
         <v>0.965034965034965</v>
       </c>
     </row>
-    <row r="9" spans="1:70">
+    <row r="9" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>77</v>
       </c>
@@ -3370,7 +3375,7 @@
         <v>0.97202797202797198</v>
       </c>
     </row>
-    <row r="10" spans="1:70">
+    <row r="10" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>77</v>
       </c>
@@ -3525,7 +3530,7 @@
         <v>0.95804195804195802</v>
       </c>
     </row>
-    <row r="11" spans="1:70">
+    <row r="11" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>185</v>
       </c>
@@ -3623,7 +3628,7 @@
         <v>0.94795539033457255</v>
       </c>
     </row>
-    <row r="12" spans="1:70">
+    <row r="12" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>185</v>
       </c>
@@ -3769,7 +3774,7 @@
         <v>0.95910780669144979</v>
       </c>
     </row>
-    <row r="13" spans="1:70">
+    <row r="13" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>185</v>
       </c>
@@ -3930,7 +3935,7 @@
         <v>0.89591078066914498</v>
       </c>
     </row>
-    <row r="14" spans="1:70">
+    <row r="14" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>185</v>
       </c>
@@ -4085,7 +4090,7 @@
         <v>0.91078066914498146</v>
       </c>
     </row>
-    <row r="15" spans="1:70">
+    <row r="15" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>185</v>
       </c>
@@ -4255,7 +4260,7 @@
         <v>0.95539033457249067</v>
       </c>
     </row>
-    <row r="16" spans="1:70">
+    <row r="16" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>185</v>
       </c>
@@ -4410,7 +4415,7 @@
         <v>0.95539033457249067</v>
       </c>
     </row>
-    <row r="17" spans="1:70">
+    <row r="17" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>185</v>
       </c>
@@ -4568,7 +4573,7 @@
         <v>0.95539033457249067</v>
       </c>
     </row>
-    <row r="18" spans="1:70">
+    <row r="18" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>185</v>
       </c>
@@ -4723,7 +4728,7 @@
         <v>0.95910780669144979</v>
       </c>
     </row>
-    <row r="19" spans="1:70">
+    <row r="19" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>210</v>
       </c>
@@ -4821,7 +4826,7 @@
         <v>0.92509363295880154</v>
       </c>
     </row>
-    <row r="20" spans="1:70">
+    <row r="20" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>210</v>
       </c>
@@ -4967,7 +4972,7 @@
         <v>0.97752808988764039</v>
       </c>
     </row>
-    <row r="21" spans="1:70">
+    <row r="21" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>210</v>
       </c>
@@ -5128,7 +5133,7 @@
         <v>0.95131086142322097</v>
       </c>
     </row>
-    <row r="22" spans="1:70">
+    <row r="22" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>210</v>
       </c>
@@ -5283,7 +5288,7 @@
         <v>0.92509363295880154</v>
       </c>
     </row>
-    <row r="23" spans="1:70">
+    <row r="23" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>210</v>
       </c>
@@ -5453,7 +5458,7 @@
         <v>0.95880149812734083</v>
       </c>
     </row>
-    <row r="24" spans="1:70">
+    <row r="24" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>210</v>
       </c>
@@ -5608,7 +5613,7 @@
         <v>0.92509363295880154</v>
       </c>
     </row>
-    <row r="25" spans="1:70">
+    <row r="25" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>210</v>
       </c>
@@ -5766,7 +5771,7 @@
         <v>0.97003745318352064</v>
       </c>
     </row>
-    <row r="26" spans="1:70">
+    <row r="26" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>210</v>
       </c>
@@ -5921,7 +5926,7 @@
         <v>0.97752808988764039</v>
       </c>
     </row>
-    <row r="27" spans="1:70">
+    <row r="27" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>77</v>
       </c>
@@ -6100,7 +6105,7 @@
         <v>0.38811188811188813</v>
       </c>
     </row>
-    <row r="28" spans="1:70">
+    <row r="28" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>77</v>
       </c>
@@ -6288,7 +6293,7 @@
         <v>0.38811188811188813</v>
       </c>
     </row>
-    <row r="29" spans="1:70">
+    <row r="29" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>185</v>
       </c>
@@ -6467,7 +6472,7 @@
         <v>0.59479553903345728</v>
       </c>
     </row>
-    <row r="30" spans="1:70">
+    <row r="30" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>185</v>
       </c>
@@ -6655,7 +6660,7 @@
         <v>0.59479553903345728</v>
       </c>
     </row>
-    <row r="31" spans="1:70">
+    <row r="31" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>210</v>
       </c>
@@ -6834,7 +6839,7 @@
         <v>0.5842696629213483</v>
       </c>
     </row>
-    <row r="32" spans="1:70">
+    <row r="32" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>210</v>
       </c>
@@ -7022,7 +7027,7 @@
         <v>0.5842696629213483</v>
       </c>
     </row>
-    <row r="33" spans="1:70">
+    <row r="33" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>279</v>
       </c>
@@ -7186,7 +7191,7 @@
         <v>0.91666666666666663</v>
       </c>
     </row>
-    <row r="34" spans="1:70">
+    <row r="34" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>279</v>
       </c>
@@ -7347,7 +7352,7 @@
         <v>0.80797101449275366</v>
       </c>
     </row>
-    <row r="35" spans="1:70">
+    <row r="35" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>279</v>
       </c>
@@ -7511,7 +7516,7 @@
         <v>0.90217391304347827</v>
       </c>
     </row>
-    <row r="36" spans="1:70">
+    <row r="36" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>279</v>
       </c>
@@ -7657,7 +7662,7 @@
         <v>0.69565217391304346</v>
       </c>
     </row>
-    <row r="37" spans="1:70">
+    <row r="37" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>77</v>
       </c>
@@ -7803,7 +7808,7 @@
         <v>0.73076923076923073</v>
       </c>
     </row>
-    <row r="38" spans="1:70">
+    <row r="38" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>185</v>
       </c>
@@ -7949,7 +7954,7 @@
         <v>0.84758364312267653</v>
       </c>
     </row>
-    <row r="39" spans="1:70">
+    <row r="39" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>210</v>
       </c>
@@ -8095,7 +8100,7 @@
         <v>0.83520599250936334</v>
       </c>
     </row>
-    <row r="40" spans="1:70">
+    <row r="40" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>338</v>
       </c>
@@ -8259,7 +8264,7 @@
         <v>0.80303030303030298</v>
       </c>
     </row>
-    <row r="41" spans="1:70">
+    <row r="41" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>338</v>
       </c>
@@ -8420,7 +8425,7 @@
         <v>0.91666666666666663</v>
       </c>
     </row>
-    <row r="42" spans="1:70">
+    <row r="42" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>279</v>
       </c>
@@ -8572,7 +8577,7 @@
         <v>0.84057971014492749</v>
       </c>
     </row>
-    <row r="43" spans="1:70">
+    <row r="43" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>279</v>
       </c>
@@ -8751,7 +8756,7 @@
         <v>0.47826086956521741</v>
       </c>
     </row>
-    <row r="44" spans="1:70">
+    <row r="44" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>279</v>
       </c>
@@ -8939,7 +8944,7 @@
         <v>0.58695652173913049</v>
       </c>
     </row>
-    <row r="45" spans="1:70">
+    <row r="45" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>373</v>
       </c>
@@ -9118,7 +9123,7 @@
         <v>0.27777777777777779</v>
       </c>
     </row>
-    <row r="46" spans="1:70">
+    <row r="46" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>373</v>
       </c>
@@ -9306,7 +9311,7 @@
         <v>0.59722222222222221</v>
       </c>
     </row>
-    <row r="47" spans="1:70">
+    <row r="47" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>373</v>
       </c>
@@ -9485,7 +9490,7 @@
         <v>0.53819444444444442</v>
       </c>
     </row>
-    <row r="48" spans="1:70">
+    <row r="48" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>373</v>
       </c>
@@ -9673,7 +9678,7 @@
         <v>0.53819444444444442</v>
       </c>
     </row>
-    <row r="49" spans="1:70">
+    <row r="49" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>393</v>
       </c>
@@ -9852,7 +9857,7 @@
         <v>0.29710144927536231</v>
       </c>
     </row>
-    <row r="50" spans="1:70">
+    <row r="50" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>393</v>
       </c>
@@ -10040,7 +10045,7 @@
         <v>0.47101449275362323</v>
       </c>
     </row>
-    <row r="51" spans="1:70">
+    <row r="51" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>406</v>
       </c>
@@ -10186,7 +10191,7 @@
         <v>0.82905982905982911</v>
       </c>
     </row>
-    <row r="52" spans="1:70">
+    <row r="52" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>406</v>
       </c>
@@ -10332,7 +10337,7 @@
         <v>0.84188034188034189</v>
       </c>
     </row>
-    <row r="53" spans="1:70">
+    <row r="53" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>416</v>
       </c>
@@ -10478,7 +10483,7 @@
         <v>0.81196581196581197</v>
       </c>
     </row>
-    <row r="54" spans="1:70">
+    <row r="54" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>422</v>
       </c>
@@ -10624,7 +10629,7 @@
         <v>0.81545064377682408</v>
       </c>
     </row>
-    <row r="55" spans="1:70">
+    <row r="55" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>428</v>
       </c>
@@ -10770,7 +10775,7 @@
         <v>0.84549356223175964</v>
       </c>
     </row>
-    <row r="56" spans="1:70">
+    <row r="56" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>435</v>
       </c>
@@ -10916,7 +10921,7 @@
         <v>0.83690987124463523</v>
       </c>
     </row>
-    <row r="57" spans="1:70">
+    <row r="57" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>442</v>
       </c>
@@ -11095,7 +11100,7 @@
         <v>0.61006289308176098</v>
       </c>
     </row>
-    <row r="58" spans="1:70">
+    <row r="58" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>442</v>
       </c>
@@ -11283,7 +11288,7 @@
         <v>0.57547169811320753</v>
       </c>
     </row>
-    <row r="59" spans="1:70">
+    <row r="59" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>338</v>
       </c>
@@ -11429,7 +11434,7 @@
         <v>0.73863636363636365</v>
       </c>
     </row>
-    <row r="60" spans="1:70">
+    <row r="60" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>406</v>
       </c>
@@ -11608,7 +11613,7 @@
         <v>0.54700854700854706</v>
       </c>
     </row>
-    <row r="61" spans="1:70">
+    <row r="61" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>406</v>
       </c>
@@ -11796,7 +11801,7 @@
         <v>0.54700854700854706</v>
       </c>
     </row>
-    <row r="62" spans="1:70">
+    <row r="62" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>406</v>
       </c>
@@ -11975,7 +11980,7 @@
         <v>0.54700854700854706</v>
       </c>
     </row>
-    <row r="63" spans="1:70">
+    <row r="63" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>406</v>
       </c>
@@ -12163,7 +12168,7 @@
         <v>0.54700854700854706</v>
       </c>
     </row>
-    <row r="64" spans="1:70">
+    <row r="64" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>416</v>
       </c>
@@ -12342,7 +12347,7 @@
         <v>0.55128205128205132</v>
       </c>
     </row>
-    <row r="65" spans="1:70">
+    <row r="65" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>416</v>
       </c>
@@ -12530,7 +12535,7 @@
         <v>0.55128205128205132</v>
       </c>
     </row>
-    <row r="66" spans="1:70">
+    <row r="66" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>422</v>
       </c>
@@ -12709,7 +12714,7 @@
         <v>0.54935622317596566</v>
       </c>
     </row>
-    <row r="67" spans="1:70">
+    <row r="67" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>422</v>
       </c>
@@ -12897,7 +12902,7 @@
         <v>0.54935622317596566</v>
       </c>
     </row>
-    <row r="68" spans="1:70">
+    <row r="68" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>428</v>
       </c>
@@ -13076,7 +13081,7 @@
         <v>0.54935622317596566</v>
       </c>
     </row>
-    <row r="69" spans="1:70">
+    <row r="69" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>428</v>
       </c>
@@ -13264,7 +13269,7 @@
         <v>0.54935622317596566</v>
       </c>
     </row>
-    <row r="70" spans="1:70">
+    <row r="70" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>435</v>
       </c>
@@ -13443,7 +13448,7 @@
         <v>0.54935622317596566</v>
       </c>
     </row>
-    <row r="71" spans="1:70">
+    <row r="71" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>435</v>
       </c>
@@ -13631,7 +13636,7 @@
         <v>0.54935622317596566</v>
       </c>
     </row>
-    <row r="72" spans="1:70">
+    <row r="72" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>338</v>
       </c>
@@ -13804,7 +13809,7 @@
         <v>0.31428571428571428</v>
       </c>
     </row>
-    <row r="73" spans="1:70">
+    <row r="73" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>489</v>
       </c>
@@ -13845,7 +13850,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="74" spans="1:70">
+    <row r="74" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>495</v>
       </c>
@@ -13886,7 +13891,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="75" spans="1:70">
+    <row r="75" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>500</v>
       </c>
@@ -13927,7 +13932,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="76" spans="1:70">
+    <row r="76" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>505</v>
       </c>
@@ -13968,7 +13973,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="77" spans="1:70">
+    <row r="77" spans="1:70" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>510</v>
       </c>

</xml_diff>